<commit_message>
Resolve the 6 rows needing review
scripts/fix-review-rows.ts: team pages from the firm's own site (direct or
Jina-rendered; portfolio redirects skipped), partner picked by Gemini from that
text and accepted only if the name is on the page; falls back to pages that
name the firm; LinkedIn via Tavily (no date filter for profiles).
- Eclipse: website eclipse.vc -> eclipse.capital (verified via /team), Lior Susan
- Kalaari: Vani Kola · LDV: Evan Nisselson · NB Ventures: Neeleshwar Bhatnagar
- Speciale: Vishesh Rajaram · Inflection Point: Vinay Bansal (team page fixed;
  /team redirected to a portfolio company)
lib/search.ts: days=0 means no date filter.
tests/db-guard: scripts/proofs.ts exempt (it attempts denied writes on purpose).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/vc-list-export.xlsx
+++ b/data/vc-list-export.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="598" uniqueCount="248">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="598" uniqueCount="253">
   <si>
     <t>Firm</t>
   </si>
@@ -152,544 +152,559 @@
     <t>NB Ventures</t>
   </si>
   <si>
+    <t>Neeleshwar Bhatnagar</t>
+  </si>
+  <si>
+    <t>GCC / India</t>
+  </si>
+  <si>
+    <t>Led Edgistify $1.4M seed (logistics tech, Jan 2026) - verify B2B software fit</t>
+  </si>
+  <si>
+    <t>https://nbventuresme.com</t>
+  </si>
+  <si>
+    <t>Nexus Venture Partners</t>
+  </si>
+  <si>
+    <t>Suvir Sujan</t>
+  </si>
+  <si>
+    <t>India / US</t>
+  </si>
+  <si>
+    <t>Backer of Delhivery; SaaS/enterprise skew; co-invests with Stellaris/Blume</t>
+  </si>
+  <si>
+    <t>https://www.nexusvp.com</t>
+  </si>
+  <si>
+    <t>Orios Venture Partners</t>
+  </si>
+  <si>
+    <t>Rehan Yar Khan</t>
+  </si>
+  <si>
+    <t>Reported to back logistics among consumer/fintech; smaller seed checks ($300K-$700K) - verify B2B fit</t>
+  </si>
+  <si>
+    <t>https://oriosvp.com</t>
+  </si>
+  <si>
+    <t>Peak XV Partners (Surge)</t>
+  </si>
+  <si>
+    <t>Rajan Anandan</t>
+  </si>
+  <si>
+    <t>India / SEA</t>
+  </si>
+  <si>
+    <t>Sequoia India's Surge led Shipsy Series A (logistics SaaS); runs seed program Surge</t>
+  </si>
+  <si>
+    <t>https://www.peakxv.com</t>
+  </si>
+  <si>
+    <t>Primary Venture Partners</t>
+  </si>
+  <si>
+    <t>Zach Fredericks</t>
+  </si>
+  <si>
+    <t>Partner Zach Fredericks discussed supply chain investing on Dynamo podcast (Dec 2024); cited as investor in Lyriq</t>
+  </si>
+  <si>
+    <t>https://www.primary.vc</t>
+  </si>
+  <si>
+    <t>Schematic Ventures</t>
+  </si>
+  <si>
+    <t>Julian Counihan</t>
+  </si>
+  <si>
+    <t>Early-stage fund for supply chain, manufacturing &amp; commerce infrastructure; GP Julian Counihan appeared on Dynamo podcast</t>
+  </si>
+  <si>
+    <t>https://www.schematicventures.com</t>
+  </si>
+  <si>
+    <t>Stellaris Venture Partners</t>
+  </si>
+  <si>
+    <t>Sayantan Sarkar</t>
+  </si>
+  <si>
+    <t>Seed to Series A; focus areas reported to include B2B SaaS and supply chain tech (single secondary source - verify on firm site)</t>
+  </si>
+  <si>
+    <t>https://www.stellarisvp.com</t>
+  </si>
+  <si>
+    <t>Z47 (Matrix Partners India)</t>
+  </si>
+  <si>
+    <t>Avnish Bajaj</t>
+  </si>
+  <si>
+    <t>Historically active in logistics; seed pace slowed in 2026 per one source - verify</t>
+  </si>
+  <si>
+    <t>https://www.z47.com</t>
+  </si>
+  <si>
+    <t>100Unicorns</t>
+  </si>
+  <si>
+    <t>Dr Apoorva Ranjan Sharma</t>
+  </si>
+  <si>
+    <t>P2</t>
+  </si>
+  <si>
+    <t>Rubric swap-in (score 16): co-led seed in 1Buy.AI (AI-powered electronics component procurement, bill of materials optimisation, and inventory liquidation; 2026-01-29)</t>
+  </si>
+  <si>
+    <t>https://100unicorns.in</t>
+  </si>
+  <si>
+    <t>3one4 Capital</t>
+  </si>
+  <si>
+    <t>Pranav Pai</t>
+  </si>
+  <si>
+    <t>Pre-seed to Series A; SaaS, fintech, consumer, AI</t>
+  </si>
+  <si>
+    <t>https://www.3one4capital.com</t>
+  </si>
+  <si>
+    <t>8VC</t>
+  </si>
+  <si>
+    <t>Jake Medwell</t>
+  </si>
+  <si>
+    <t>Cited as most active freight-tech investor per PitchBook (via Ellty); multi-stage</t>
+  </si>
+  <si>
+    <t>https://8vc.com</t>
+  </si>
+  <si>
+    <t>Accel India</t>
+  </si>
+  <si>
+    <t>Subrata Mitra</t>
+  </si>
+  <si>
+    <t>Among most active seed investors globally (59 deals/12 mo per ALTSS); SaaS focus</t>
+  </si>
+  <si>
+    <t>https://www.accel.com</t>
+  </si>
+  <si>
+    <t>Arali Ventures</t>
+  </si>
+  <si>
+    <t>Arun Raghavan</t>
+  </si>
+  <si>
+    <t>AI/B2B software seed fund</t>
+  </si>
+  <si>
+    <t>https://www.araliventures.in</t>
+  </si>
+  <si>
+    <t>Better Capital</t>
+  </si>
+  <si>
+    <t>Vaibhav Domkundwar</t>
+  </si>
+  <si>
+    <t>Listed among top B2B VC funds in India</t>
+  </si>
+  <si>
+    <t>https://www.bettercapital.vc</t>
+  </si>
+  <si>
+    <t>Blume Ventures</t>
+  </si>
+  <si>
+    <t>Sanjay Nath</t>
+  </si>
+  <si>
+    <t>Among most active India seed investors (24 seed deals in 12 months per ALTSS ranking); SaaS, fintech, consumer, deeptech</t>
+  </si>
+  <si>
+    <t>https://blume.vc</t>
+  </si>
+  <si>
+    <t>Chicago Ventures</t>
+  </si>
+  <si>
+    <t>Stuart Larkins</t>
+  </si>
+  <si>
+    <t>Named logistics specialist</t>
+  </si>
+  <si>
+    <t>https://www.chicagoventures.com</t>
+  </si>
+  <si>
+    <t>Chiratae Ventures</t>
+  </si>
+  <si>
+    <t>TC Meenakshisundaram</t>
+  </si>
+  <si>
+    <t>Rubric swap-in (score 40.6): led seed-extension in ContraVault AI (AI-powered procurement intelligence and tender bidding software; 2026-06-16)</t>
+  </si>
+  <si>
+    <t>https://www.chiratae.com</t>
+  </si>
+  <si>
+    <t>Elevation Capital</t>
+  </si>
+  <si>
+    <t>Ravi Adusumalli</t>
+  </si>
+  <si>
+    <t>Active at seed alongside later stages; consumer, fintech, SaaS</t>
+  </si>
+  <si>
+    <t>https://www.elevationcapital.com</t>
+  </si>
+  <si>
+    <t>Fuel Ventures</t>
+  </si>
+  <si>
+    <t>Mark Pearson</t>
+  </si>
+  <si>
+    <t>Named among supply-chain/logistics active VCs</t>
+  </si>
+  <si>
+    <t>https://www.fuel.ventures</t>
+  </si>
+  <si>
+    <t>Inflection Point Ventures</t>
+  </si>
+  <si>
+    <t>Vinay Bansal</t>
+  </si>
+  <si>
+    <t>30 seed deals in 12 months (ALTSS); 2026 logistics deal Daakit was consumer logistics - adjacent</t>
+  </si>
+  <si>
+    <t>https://ipventures.in</t>
+  </si>
+  <si>
+    <t>Kalaari Capital</t>
+  </si>
+  <si>
+    <t>Vani Kola</t>
+  </si>
+  <si>
+    <t>Leads early-stage deal volume in India; consumer, B2B, AI/SaaS</t>
+  </si>
+  <si>
+    <t>https://kalaari.com</t>
+  </si>
+  <si>
+    <t>Lightspeed India</t>
+  </si>
+  <si>
+    <t>Bejul Somaia</t>
+  </si>
+  <si>
+    <t>Active in SaaS/AI/enterprise</t>
+  </si>
+  <si>
+    <t>https://lsvp.com</t>
+  </si>
+  <si>
+    <t>Mu Ventures</t>
+  </si>
+  <si>
+    <t>Gary Benerofe</t>
+  </si>
+  <si>
+    <t>Listed among pre-seed/seed supply chain funds</t>
+  </si>
+  <si>
+    <t>https://www.muventures.com</t>
+  </si>
+  <si>
+    <t>Overlay Capital</t>
+  </si>
+  <si>
+    <t>Chadd Evans</t>
+  </si>
+  <si>
+    <t>https://overlaycapital.com</t>
+  </si>
+  <si>
+    <t>Pentathlon Ventures</t>
+  </si>
+  <si>
+    <t>Madhukar Bhatia</t>
+  </si>
+  <si>
+    <t>Rubric swap-in (score 21.9): led pre-seed in SuperProcure (Unified TMS and freight lifecycle management software; 2026-02-25)</t>
+  </si>
+  <si>
+    <t>https://pentathlon.vc</t>
+  </si>
+  <si>
+    <t>Picus Capital</t>
+  </si>
+  <si>
+    <t>Florian Reichert</t>
+  </si>
+  <si>
+    <t>Global (Germany)</t>
+  </si>
+  <si>
+    <t>Rubric swap-in (score 42.4): led seed in Compri (AI-powered procurement software for industrial companies; 2026-06-24)</t>
+  </si>
+  <si>
+    <t>https://www.picuscap.com</t>
+  </si>
+  <si>
+    <t>Prime Venture Partners</t>
+  </si>
+  <si>
+    <t>Amit Somani</t>
+  </si>
+  <si>
+    <t>Bengaluru B2B SaaS/fintech seed fund; reported $1M-$4M first cheques</t>
+  </si>
+  <si>
+    <t>https://www.primevp.in</t>
+  </si>
+  <si>
+    <t>Supply Change Capital</t>
+  </si>
+  <si>
+    <t>Shayna Harris</t>
+  </si>
+  <si>
+    <t>Appears in Signal NFX supply-chain tech seed investor list</t>
+  </si>
+  <si>
+    <t>https://supplychange.fund</t>
+  </si>
+  <si>
+    <t>Susa Ventures</t>
+  </si>
+  <si>
+    <t>Seth Berman</t>
+  </si>
+  <si>
+    <t>https://susaventures.com</t>
+  </si>
+  <si>
+    <t>Tech Square Ventures</t>
+  </si>
+  <si>
+    <t>Blake Patton</t>
+  </si>
+  <si>
+    <t>Listed among pre-seed/seed logistics funds</t>
+  </si>
+  <si>
+    <t>https://techsquareventures.com</t>
+  </si>
+  <si>
+    <t>Titan Capital</t>
+  </si>
+  <si>
+    <t>Rohit Bansal</t>
+  </si>
+  <si>
+    <t>Listed among top B2B VC funds in India (software, IT)</t>
+  </si>
+  <si>
+    <t>https://titancapital.vc</t>
+  </si>
+  <si>
+    <t>Turbostart</t>
+  </si>
+  <si>
+    <t>Rajagopal Koushik</t>
+  </si>
+  <si>
+    <t>Rubric swap-in (score 25.3): co-led seed-extension in Lawyered (legal infrastructure and proactive compliance platform for mobility and logistics; 2026-04-21)</t>
+  </si>
+  <si>
+    <t>https://turbostart.co</t>
+  </si>
+  <si>
+    <t>Wavemaker Partners</t>
+  </si>
+  <si>
+    <t>Paul Santos</t>
+  </si>
+  <si>
+    <t>Rubric swap-in (score 23.7): led pre-seed in Confluxe (Platform providing market entry strategy, digital commerce, merchandising, and supply chain operations; 2026-03-11)</t>
+  </si>
+  <si>
+    <t>https://wavemaker.vc</t>
+  </si>
+  <si>
+    <t>YourNest Venture Capital</t>
+  </si>
+  <si>
+    <t>Girish Shivani</t>
+  </si>
+  <si>
+    <t>Rubric swap-in (score 42.4): led seed in CargoFL (logistics technology platform to optimize freight and supply chain operations; 2026-06-24)</t>
+  </si>
+  <si>
+    <t>https://yournest.in</t>
+  </si>
+  <si>
+    <t>100X.VC</t>
+  </si>
+  <si>
+    <t>Sanjay Mehta</t>
+  </si>
+  <si>
+    <t>P3</t>
+  </si>
+  <si>
+    <t>Active India seed fund (iSAFE structure)</t>
+  </si>
+  <si>
+    <t>https://www.100x.vc</t>
+  </si>
+  <si>
+    <t>Ankur Capital</t>
+  </si>
+  <si>
+    <t>Krishnan Neelakantan</t>
+  </si>
+  <si>
+    <t>Agritech/agri-supply-chain focus - adjacent</t>
+  </si>
+  <si>
+    <t>https://www.ankurcapital.com</t>
+  </si>
+  <si>
+    <t>Antler India</t>
+  </si>
+  <si>
+    <t>Nitin Sharma</t>
+  </si>
+  <si>
+    <t>Day-zero/pre-seed platform</t>
+  </si>
+  <si>
+    <t>https://www.antler.co</t>
+  </si>
+  <si>
+    <t>Eclipse Ventures</t>
+  </si>
+  <si>
+    <t>Lior Susan</t>
+  </si>
+  <si>
+    <t>Listed for logistics but industrial/hardware-heavy - likely adjacent, not B2B software</t>
+  </si>
+  <si>
+    <t>https://eclipse.capital</t>
+  </si>
+  <si>
+    <t>LDV Capital</t>
+  </si>
+  <si>
+    <t>Evan Nisselson</t>
+  </si>
+  <si>
+    <t>Listed among early-stage logistics funds (deep-tech/visual tech skew)</t>
+  </si>
+  <si>
+    <t>https://www.ldv.co</t>
+  </si>
+  <si>
+    <t>Navigate Ventures</t>
+  </si>
+  <si>
+    <t>Ivan Nikkhoo</t>
+  </si>
+  <si>
+    <t>Appears in Signal NFX supply-chain seed list (LA region); confirm still active</t>
+  </si>
+  <si>
+    <t>https://www.navigatevc.com</t>
+  </si>
+  <si>
+    <t>pi Ventures</t>
+  </si>
+  <si>
+    <t>Shubham Sandeep</t>
+  </si>
+  <si>
+    <t>Deep-tech/AI focus - likely thematic (AI) rather than logistics</t>
+  </si>
+  <si>
+    <t>https://www.piventures.in</t>
+  </si>
+  <si>
+    <t>Prologis Ventures</t>
+  </si>
+  <si>
+    <t>William O'Donnell</t>
+  </si>
+  <si>
+    <t>Global</t>
+  </si>
+  <si>
+    <t>Corporate VC of a warehousing REIT; track for thematic signals</t>
+  </si>
+  <si>
+    <t>https://www.prologis.com</t>
+  </si>
+  <si>
+    <t>Speciale Invest</t>
+  </si>
+  <si>
+    <t>Vishesh Rajaram</t>
+  </si>
+  <si>
+    <t>Deep-tech/space/robotics focus; Rs 600Cr Fund III (Aug 2025) - mostly adjacent for B2B SaaS</t>
+  </si>
+  <si>
+    <t>https://www.specialeinvest.com</t>
+  </si>
+  <si>
+    <t>TMV</t>
+  </si>
+  <si>
+    <t>Marina Hadjipateras</t>
+  </si>
+  <si>
+    <t>Listed among early-stage logistics funds</t>
+  </si>
+  <si>
+    <t>https://www.tmv.vc</t>
+  </si>
+  <si>
+    <t>Archived reason</t>
+  </si>
+  <si>
+    <t>Enrission India Capital</t>
+  </si>
+  <si>
+    <t>YUSUKE KAKIMOTO</t>
+  </si>
+  <si>
+    <t>Led Hexalog $4M seed (logistics tech, Jan 2026) - verify B2B software fit</t>
+  </si>
+  <si>
     <t/>
-  </si>
-  <si>
-    <t>GCC / India</t>
-  </si>
-  <si>
-    <t>Led Edgistify $1.4M seed (logistics tech, Jan 2026) - verify B2B software fit</t>
-  </si>
-  <si>
-    <t>https://nbventuresme.com</t>
-  </si>
-  <si>
-    <t>Nexus Venture Partners</t>
-  </si>
-  <si>
-    <t>Suvir Sujan</t>
-  </si>
-  <si>
-    <t>India / US</t>
-  </si>
-  <si>
-    <t>Backer of Delhivery; SaaS/enterprise skew; co-invests with Stellaris/Blume</t>
-  </si>
-  <si>
-    <t>https://www.nexusvp.com</t>
-  </si>
-  <si>
-    <t>Orios Venture Partners</t>
-  </si>
-  <si>
-    <t>Rehan Yar Khan</t>
-  </si>
-  <si>
-    <t>Reported to back logistics among consumer/fintech; smaller seed checks ($300K-$700K) - verify B2B fit</t>
-  </si>
-  <si>
-    <t>https://oriosvp.com</t>
-  </si>
-  <si>
-    <t>Peak XV Partners (Surge)</t>
-  </si>
-  <si>
-    <t>Rajan Anandan</t>
-  </si>
-  <si>
-    <t>India / SEA</t>
-  </si>
-  <si>
-    <t>Sequoia India's Surge led Shipsy Series A (logistics SaaS); runs seed program Surge</t>
-  </si>
-  <si>
-    <t>https://www.peakxv.com</t>
-  </si>
-  <si>
-    <t>Primary Venture Partners</t>
-  </si>
-  <si>
-    <t>Zach Fredericks</t>
-  </si>
-  <si>
-    <t>Partner Zach Fredericks discussed supply chain investing on Dynamo podcast (Dec 2024); cited as investor in Lyriq</t>
-  </si>
-  <si>
-    <t>https://www.primary.vc</t>
-  </si>
-  <si>
-    <t>Schematic Ventures</t>
-  </si>
-  <si>
-    <t>Julian Counihan</t>
-  </si>
-  <si>
-    <t>Early-stage fund for supply chain, manufacturing &amp; commerce infrastructure; GP Julian Counihan appeared on Dynamo podcast</t>
-  </si>
-  <si>
-    <t>https://www.schematicventures.com</t>
-  </si>
-  <si>
-    <t>Stellaris Venture Partners</t>
-  </si>
-  <si>
-    <t>Sayantan Sarkar</t>
-  </si>
-  <si>
-    <t>Seed to Series A; focus areas reported to include B2B SaaS and supply chain tech (single secondary source - verify on firm site)</t>
-  </si>
-  <si>
-    <t>https://www.stellarisvp.com</t>
-  </si>
-  <si>
-    <t>Z47 (Matrix Partners India)</t>
-  </si>
-  <si>
-    <t>Avnish Bajaj</t>
-  </si>
-  <si>
-    <t>Historically active in logistics; seed pace slowed in 2026 per one source - verify</t>
-  </si>
-  <si>
-    <t>https://www.z47.com</t>
-  </si>
-  <si>
-    <t>100Unicorns</t>
-  </si>
-  <si>
-    <t>Dr Apoorva Ranjan Sharma</t>
-  </si>
-  <si>
-    <t>P2</t>
-  </si>
-  <si>
-    <t>Rubric swap-in (score 16): co-led seed in 1Buy.AI (AI-powered electronics component procurement, bill of materials optimisation, and inventory liquidation; 2026-01-29)</t>
-  </si>
-  <si>
-    <t>https://100unicorns.in</t>
-  </si>
-  <si>
-    <t>3one4 Capital</t>
-  </si>
-  <si>
-    <t>Pranav Pai</t>
-  </si>
-  <si>
-    <t>Pre-seed to Series A; SaaS, fintech, consumer, AI</t>
-  </si>
-  <si>
-    <t>https://www.3one4capital.com</t>
-  </si>
-  <si>
-    <t>8VC</t>
-  </si>
-  <si>
-    <t>Jake Medwell</t>
-  </si>
-  <si>
-    <t>Cited as most active freight-tech investor per PitchBook (via Ellty); multi-stage</t>
-  </si>
-  <si>
-    <t>https://8vc.com</t>
-  </si>
-  <si>
-    <t>Accel India</t>
-  </si>
-  <si>
-    <t>Subrata Mitra</t>
-  </si>
-  <si>
-    <t>Among most active seed investors globally (59 deals/12 mo per ALTSS); SaaS focus</t>
-  </si>
-  <si>
-    <t>https://www.accel.com</t>
-  </si>
-  <si>
-    <t>Arali Ventures</t>
-  </si>
-  <si>
-    <t>Arun Raghavan</t>
-  </si>
-  <si>
-    <t>AI/B2B software seed fund</t>
-  </si>
-  <si>
-    <t>https://www.araliventures.in</t>
-  </si>
-  <si>
-    <t>Better Capital</t>
-  </si>
-  <si>
-    <t>Vaibhav Domkundwar</t>
-  </si>
-  <si>
-    <t>Listed among top B2B VC funds in India</t>
-  </si>
-  <si>
-    <t>https://www.bettercapital.vc</t>
-  </si>
-  <si>
-    <t>Blume Ventures</t>
-  </si>
-  <si>
-    <t>Sanjay Nath</t>
-  </si>
-  <si>
-    <t>Among most active India seed investors (24 seed deals in 12 months per ALTSS ranking); SaaS, fintech, consumer, deeptech</t>
-  </si>
-  <si>
-    <t>https://blume.vc</t>
-  </si>
-  <si>
-    <t>Chicago Ventures</t>
-  </si>
-  <si>
-    <t>Stuart Larkins</t>
-  </si>
-  <si>
-    <t>Named logistics specialist</t>
-  </si>
-  <si>
-    <t>https://www.chicagoventures.com</t>
-  </si>
-  <si>
-    <t>Chiratae Ventures</t>
-  </si>
-  <si>
-    <t>TC Meenakshisundaram</t>
-  </si>
-  <si>
-    <t>Rubric swap-in (score 40.6): led seed-extension in ContraVault AI (AI-powered procurement intelligence and tender bidding software; 2026-06-16)</t>
-  </si>
-  <si>
-    <t>https://www.chiratae.com</t>
-  </si>
-  <si>
-    <t>Elevation Capital</t>
-  </si>
-  <si>
-    <t>Ravi Adusumalli</t>
-  </si>
-  <si>
-    <t>Active at seed alongside later stages; consumer, fintech, SaaS</t>
-  </si>
-  <si>
-    <t>https://www.elevationcapital.com</t>
-  </si>
-  <si>
-    <t>Fuel Ventures</t>
-  </si>
-  <si>
-    <t>Mark Pearson</t>
-  </si>
-  <si>
-    <t>Named among supply-chain/logistics active VCs</t>
-  </si>
-  <si>
-    <t>https://www.fuel.ventures</t>
-  </si>
-  <si>
-    <t>Inflection Point Ventures</t>
-  </si>
-  <si>
-    <t>30 seed deals in 12 months (ALTSS); 2026 logistics deal Daakit was consumer logistics - adjacent</t>
-  </si>
-  <si>
-    <t>https://ipventures.in</t>
-  </si>
-  <si>
-    <t>Kalaari Capital</t>
-  </si>
-  <si>
-    <t>Leads early-stage deal volume in India; consumer, B2B, AI/SaaS</t>
-  </si>
-  <si>
-    <t>https://kalaari.com</t>
-  </si>
-  <si>
-    <t>Lightspeed India</t>
-  </si>
-  <si>
-    <t>Bejul Somaia</t>
-  </si>
-  <si>
-    <t>Active in SaaS/AI/enterprise</t>
-  </si>
-  <si>
-    <t>https://lsvp.com</t>
-  </si>
-  <si>
-    <t>Mu Ventures</t>
-  </si>
-  <si>
-    <t>Gary Benerofe</t>
-  </si>
-  <si>
-    <t>Listed among pre-seed/seed supply chain funds</t>
-  </si>
-  <si>
-    <t>https://www.muventures.com</t>
-  </si>
-  <si>
-    <t>Overlay Capital</t>
-  </si>
-  <si>
-    <t>Chadd Evans</t>
-  </si>
-  <si>
-    <t>https://overlaycapital.com</t>
-  </si>
-  <si>
-    <t>Pentathlon Ventures</t>
-  </si>
-  <si>
-    <t>Madhukar Bhatia</t>
-  </si>
-  <si>
-    <t>Rubric swap-in (score 21.9): led pre-seed in SuperProcure (Unified TMS and freight lifecycle management software; 2026-02-25)</t>
-  </si>
-  <si>
-    <t>https://pentathlon.vc</t>
-  </si>
-  <si>
-    <t>Picus Capital</t>
-  </si>
-  <si>
-    <t>Florian Reichert</t>
-  </si>
-  <si>
-    <t>Global (Germany)</t>
-  </si>
-  <si>
-    <t>Rubric swap-in (score 42.4): led seed in Compri (AI-powered procurement software for industrial companies; 2026-06-24)</t>
-  </si>
-  <si>
-    <t>https://www.picuscap.com</t>
-  </si>
-  <si>
-    <t>Prime Venture Partners</t>
-  </si>
-  <si>
-    <t>Amit Somani</t>
-  </si>
-  <si>
-    <t>Bengaluru B2B SaaS/fintech seed fund; reported $1M-$4M first cheques</t>
-  </si>
-  <si>
-    <t>https://www.primevp.in</t>
-  </si>
-  <si>
-    <t>Supply Change Capital</t>
-  </si>
-  <si>
-    <t>Shayna Harris</t>
-  </si>
-  <si>
-    <t>Appears in Signal NFX supply-chain tech seed investor list</t>
-  </si>
-  <si>
-    <t>https://supplychange.fund</t>
-  </si>
-  <si>
-    <t>Susa Ventures</t>
-  </si>
-  <si>
-    <t>Seth Berman</t>
-  </si>
-  <si>
-    <t>https://susaventures.com</t>
-  </si>
-  <si>
-    <t>Tech Square Ventures</t>
-  </si>
-  <si>
-    <t>Blake Patton</t>
-  </si>
-  <si>
-    <t>Listed among pre-seed/seed logistics funds</t>
-  </si>
-  <si>
-    <t>https://techsquareventures.com</t>
-  </si>
-  <si>
-    <t>Titan Capital</t>
-  </si>
-  <si>
-    <t>Rohit Bansal</t>
-  </si>
-  <si>
-    <t>Listed among top B2B VC funds in India (software, IT)</t>
-  </si>
-  <si>
-    <t>https://titancapital.vc</t>
-  </si>
-  <si>
-    <t>Turbostart</t>
-  </si>
-  <si>
-    <t>Rajagopal Koushik</t>
-  </si>
-  <si>
-    <t>Rubric swap-in (score 25.3): co-led seed-extension in Lawyered (legal infrastructure and proactive compliance platform for mobility and logistics; 2026-04-21)</t>
-  </si>
-  <si>
-    <t>https://turbostart.co</t>
-  </si>
-  <si>
-    <t>Wavemaker Partners</t>
-  </si>
-  <si>
-    <t>Paul Santos</t>
-  </si>
-  <si>
-    <t>Rubric swap-in (score 23.7): led pre-seed in Confluxe (Platform providing market entry strategy, digital commerce, merchandising, and supply chain operations; 2026-03-11)</t>
-  </si>
-  <si>
-    <t>https://wavemaker.vc</t>
-  </si>
-  <si>
-    <t>YourNest Venture Capital</t>
-  </si>
-  <si>
-    <t>Girish Shivani</t>
-  </si>
-  <si>
-    <t>Rubric swap-in (score 42.4): led seed in CargoFL (logistics technology platform to optimize freight and supply chain operations; 2026-06-24)</t>
-  </si>
-  <si>
-    <t>https://yournest.in</t>
-  </si>
-  <si>
-    <t>100X.VC</t>
-  </si>
-  <si>
-    <t>Sanjay Mehta</t>
-  </si>
-  <si>
-    <t>P3</t>
-  </si>
-  <si>
-    <t>Active India seed fund (iSAFE structure)</t>
-  </si>
-  <si>
-    <t>https://www.100x.vc</t>
-  </si>
-  <si>
-    <t>Ankur Capital</t>
-  </si>
-  <si>
-    <t>Krishnan Neelakantan</t>
-  </si>
-  <si>
-    <t>Agritech/agri-supply-chain focus - adjacent</t>
-  </si>
-  <si>
-    <t>https://www.ankurcapital.com</t>
-  </si>
-  <si>
-    <t>Antler India</t>
-  </si>
-  <si>
-    <t>Nitin Sharma</t>
-  </si>
-  <si>
-    <t>Day-zero/pre-seed platform</t>
-  </si>
-  <si>
-    <t>https://www.antler.co</t>
-  </si>
-  <si>
-    <t>Eclipse Ventures</t>
-  </si>
-  <si>
-    <t>Lior Susan</t>
-  </si>
-  <si>
-    <t>Listed for logistics but industrial/hardware-heavy - likely adjacent, not B2B software</t>
-  </si>
-  <si>
-    <t>https://ventureequity.eclipse.vc</t>
-  </si>
-  <si>
-    <t>LDV Capital</t>
-  </si>
-  <si>
-    <t>Listed among early-stage logistics funds (deep-tech/visual tech skew)</t>
-  </si>
-  <si>
-    <t>https://www.ldv.co</t>
-  </si>
-  <si>
-    <t>Navigate Ventures</t>
-  </si>
-  <si>
-    <t>Ivan Nikkhoo</t>
-  </si>
-  <si>
-    <t>Appears in Signal NFX supply-chain seed list (LA region); confirm still active</t>
-  </si>
-  <si>
-    <t>https://www.navigatevc.com</t>
-  </si>
-  <si>
-    <t>pi Ventures</t>
-  </si>
-  <si>
-    <t>Shubham Sandeep</t>
-  </si>
-  <si>
-    <t>Deep-tech/AI focus - likely thematic (AI) rather than logistics</t>
-  </si>
-  <si>
-    <t>https://www.piventures.in</t>
-  </si>
-  <si>
-    <t>Prologis Ventures</t>
-  </si>
-  <si>
-    <t>William O'Donnell</t>
-  </si>
-  <si>
-    <t>Global</t>
-  </si>
-  <si>
-    <t>Corporate VC of a warehousing REIT; track for thematic signals</t>
-  </si>
-  <si>
-    <t>https://www.prologis.com</t>
-  </si>
-  <si>
-    <t>Speciale Invest</t>
-  </si>
-  <si>
-    <t>Deep-tech/space/robotics focus; Rs 600Cr Fund III (Aug 2025) - mostly adjacent for B2B SaaS</t>
-  </si>
-  <si>
-    <t>https://www.specialeinvest.com</t>
-  </si>
-  <si>
-    <t>TMV</t>
-  </si>
-  <si>
-    <t>Marina Hadjipateras</t>
-  </si>
-  <si>
-    <t>Listed among early-stage logistics funds</t>
-  </si>
-  <si>
-    <t>https://www.tmv.vc</t>
-  </si>
-  <si>
-    <t>Archived reason</t>
-  </si>
-  <si>
-    <t>Enrission India Capital</t>
-  </si>
-  <si>
-    <t>YUSUKE KAKIMOTO</t>
-  </si>
-  <si>
-    <t>Led Hexalog $4M seed (logistics tech, Jan 2026) - verify B2B software fit</t>
   </si>
   <si>
     <t>yes</t>
@@ -1993,7 +2008,7 @@
         <v>125</v>
       </c>
       <c r="B27" t="s">
-        <v>46</v>
+        <v>126</v>
       </c>
       <c r="C27" t="s">
         <v>22</v>
@@ -2011,10 +2026,10 @@
         <v>23</v>
       </c>
       <c r="H27" s="1" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="I27" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="J27" t="s">
         <v>19</v>
@@ -2022,10 +2037,10 @@
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B28" t="s">
-        <v>46</v>
+        <v>130</v>
       </c>
       <c r="C28" t="s">
         <v>22</v>
@@ -2043,10 +2058,10 @@
         <v>23</v>
       </c>
       <c r="H28" s="1" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="I28" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="J28" t="s">
         <v>19</v>
@@ -2054,10 +2069,10 @@
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B29" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="C29" t="s">
         <v>22</v>
@@ -2075,10 +2090,10 @@
         <v>23</v>
       </c>
       <c r="H29" s="1" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="I29" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="J29" t="s">
         <v>19</v>
@@ -2086,10 +2101,10 @@
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B30" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="C30" t="s">
         <v>12</v>
@@ -2107,10 +2122,10 @@
         <v>29</v>
       </c>
       <c r="H30" s="1" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="I30" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="J30" t="s">
         <v>19</v>
@@ -2118,10 +2133,10 @@
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B31" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="C31" t="s">
         <v>12</v>
@@ -2142,7 +2157,7 @@
         <v>111</v>
       </c>
       <c r="I31" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="J31" t="s">
         <v>19</v>
@@ -2150,10 +2165,10 @@
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="B32" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="C32" t="s">
         <v>22</v>
@@ -2171,10 +2186,10 @@
         <v>29</v>
       </c>
       <c r="H32" s="1" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="I32" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="J32" t="s">
         <v>19</v>
@@ -2182,13 +2197,13 @@
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="B33" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="C33" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="D33" t="s">
         <v>82</v>
@@ -2203,10 +2218,10 @@
         <v>29</v>
       </c>
       <c r="H33" s="1" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="I33" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="J33" t="s">
         <v>19</v>
@@ -2214,10 +2229,10 @@
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="B34" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="C34" t="s">
         <v>22</v>
@@ -2235,10 +2250,10 @@
         <v>23</v>
       </c>
       <c r="H34" s="1" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="I34" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="J34" t="s">
         <v>19</v>
@@ -2246,10 +2261,10 @@
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="B35" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="C35" t="s">
         <v>12</v>
@@ -2267,10 +2282,10 @@
         <v>29</v>
       </c>
       <c r="H35" s="1" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="I35" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="J35" t="s">
         <v>19</v>
@@ -2278,10 +2293,10 @@
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="B36" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="C36" t="s">
         <v>12</v>
@@ -2302,7 +2317,7 @@
         <v>111</v>
       </c>
       <c r="I36" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="J36" t="s">
         <v>19</v>
@@ -2310,10 +2325,10 @@
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B37" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="C37" t="s">
         <v>12</v>
@@ -2331,10 +2346,10 @@
         <v>29</v>
       </c>
       <c r="H37" s="1" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="I37" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="J37" t="s">
         <v>19</v>
@@ -2342,10 +2357,10 @@
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B38" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="C38" t="s">
         <v>22</v>
@@ -2363,10 +2378,10 @@
         <v>29</v>
       </c>
       <c r="H38" s="1" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="I38" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="J38" t="s">
         <v>19</v>
@@ -2374,10 +2389,10 @@
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="B39" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="C39" t="s">
         <v>22</v>
@@ -2395,10 +2410,10 @@
         <v>23</v>
       </c>
       <c r="H39" s="1" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="I39" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="J39" t="s">
         <v>19</v>
@@ -2406,10 +2421,10 @@
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="B40" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="C40" t="s">
         <v>22</v>
@@ -2427,10 +2442,10 @@
         <v>23</v>
       </c>
       <c r="H40" s="1" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="I40" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="J40" t="s">
         <v>19</v>
@@ -2438,10 +2453,10 @@
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="B41" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="C41" t="s">
         <v>22</v>
@@ -2459,10 +2474,10 @@
         <v>23</v>
       </c>
       <c r="H41" s="1" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="I41" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="J41" t="s">
         <v>19</v>
@@ -2470,16 +2485,16 @@
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="B42" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="C42" t="s">
         <v>22</v>
       </c>
       <c r="D42" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="E42" t="s">
         <v>14</v>
@@ -2491,10 +2506,10 @@
         <v>23</v>
       </c>
       <c r="H42" s="1" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="I42" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="J42" t="s">
         <v>19</v>
@@ -2502,16 +2517,16 @@
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="B43" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="C43" t="s">
         <v>22</v>
       </c>
       <c r="D43" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="E43" t="s">
         <v>14</v>
@@ -2523,10 +2538,10 @@
         <v>29</v>
       </c>
       <c r="H43" s="1" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="I43" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="J43" t="s">
         <v>19</v>
@@ -2534,16 +2549,16 @@
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="B44" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="C44" t="s">
         <v>61</v>
       </c>
       <c r="D44" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="E44" t="s">
         <v>14</v>
@@ -2555,10 +2570,10 @@
         <v>23</v>
       </c>
       <c r="H44" s="1" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="I44" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="J44" t="s">
         <v>19</v>
@@ -2566,16 +2581,16 @@
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="B45" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="C45" t="s">
         <v>12</v>
       </c>
       <c r="D45" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="E45" t="s">
         <v>14</v>
@@ -2587,10 +2602,10 @@
         <v>29</v>
       </c>
       <c r="H45" s="1" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="I45" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="J45" t="s">
         <v>19</v>
@@ -2598,16 +2613,16 @@
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="B46" t="s">
-        <v>46</v>
+        <v>202</v>
       </c>
       <c r="C46" t="s">
         <v>12</v>
       </c>
       <c r="D46" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="E46" t="s">
         <v>14</v>
@@ -2619,10 +2634,10 @@
         <v>29</v>
       </c>
       <c r="H46" s="1" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="I46" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="J46" t="s">
         <v>19</v>
@@ -2630,16 +2645,16 @@
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="B47" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="C47" t="s">
         <v>12</v>
       </c>
       <c r="D47" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="E47" t="s">
         <v>28</v>
@@ -2651,10 +2666,10 @@
         <v>29</v>
       </c>
       <c r="H47" s="1" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="I47" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="J47" t="s">
         <v>19</v>
@@ -2662,16 +2677,16 @@
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="B48" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="C48" t="s">
         <v>22</v>
       </c>
       <c r="D48" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="E48" t="s">
         <v>14</v>
@@ -2683,10 +2698,10 @@
         <v>23</v>
       </c>
       <c r="H48" s="1" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="I48" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="J48" t="s">
         <v>19</v>
@@ -2694,16 +2709,16 @@
     </row>
     <row r="49" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="B49" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="C49" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="D49" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="E49" t="s">
         <v>14</v>
@@ -2715,10 +2730,10 @@
         <v>29</v>
       </c>
       <c r="H49" s="1" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="I49" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="J49" t="s">
         <v>19</v>
@@ -2726,16 +2741,16 @@
     </row>
     <row r="50" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="B50" t="s">
-        <v>46</v>
+        <v>219</v>
       </c>
       <c r="C50" t="s">
         <v>22</v>
       </c>
       <c r="D50" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="E50" t="s">
         <v>28</v>
@@ -2747,10 +2762,10 @@
         <v>23</v>
       </c>
       <c r="H50" s="1" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
       <c r="I50" t="s">
-        <v>217</v>
+        <v>221</v>
       </c>
       <c r="J50" t="s">
         <v>19</v>
@@ -2758,16 +2773,16 @@
     </row>
     <row r="51" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
       <c r="B51" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="C51" t="s">
         <v>12</v>
       </c>
       <c r="D51" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="E51" t="s">
         <v>28</v>
@@ -2779,10 +2794,10 @@
         <v>29</v>
       </c>
       <c r="H51" s="1" t="s">
-        <v>220</v>
+        <v>224</v>
       </c>
       <c r="I51" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="J51" t="s">
         <v>19</v>
@@ -2844,15 +2859,15 @@
         <v>9</v>
       </c>
       <c r="K1" s="2" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>223</v>
+        <v>227</v>
       </c>
       <c r="B2" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="C2" t="s">
         <v>22</v>
@@ -2870,24 +2885,24 @@
         <v>23</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>225</v>
+        <v>229</v>
       </c>
       <c r="I2" t="s">
-        <v>46</v>
+        <v>230</v>
       </c>
       <c r="J2" t="s">
-        <v>226</v>
+        <v>231</v>
       </c>
       <c r="K2" t="s">
-        <v>227</v>
+        <v>232</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>228</v>
+        <v>233</v>
       </c>
       <c r="B3" t="s">
-        <v>229</v>
+        <v>234</v>
       </c>
       <c r="C3" t="s">
         <v>22</v>
@@ -2899,30 +2914,30 @@
         <v>28</v>
       </c>
       <c r="F3" t="s">
-        <v>230</v>
+        <v>235</v>
       </c>
       <c r="G3" t="s">
         <v>23</v>
       </c>
       <c r="H3" s="1" t="s">
+        <v>236</v>
+      </c>
+      <c r="I3" t="s">
+        <v>237</v>
+      </c>
+      <c r="J3" t="s">
         <v>231</v>
       </c>
-      <c r="I3" t="s">
-        <v>232</v>
-      </c>
-      <c r="J3" t="s">
-        <v>226</v>
-      </c>
       <c r="K3" t="s">
-        <v>233</v>
+        <v>238</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>234</v>
+        <v>239</v>
       </c>
       <c r="B4" t="s">
-        <v>46</v>
+        <v>230</v>
       </c>
       <c r="C4" t="s">
         <v>22</v>
@@ -2940,65 +2955,65 @@
         <v>29</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>235</v>
+        <v>240</v>
       </c>
       <c r="I4" t="s">
-        <v>46</v>
+        <v>230</v>
       </c>
       <c r="J4" t="s">
-        <v>226</v>
+        <v>231</v>
       </c>
       <c r="K4" t="s">
-        <v>227</v>
+        <v>232</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>236</v>
+        <v>241</v>
       </c>
       <c r="B5" t="s">
-        <v>237</v>
+        <v>242</v>
       </c>
       <c r="C5" t="s">
         <v>22</v>
       </c>
       <c r="D5" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="E5" t="s">
         <v>14</v>
       </c>
       <c r="F5" t="s">
-        <v>230</v>
+        <v>235</v>
       </c>
       <c r="G5" t="s">
         <v>23</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>238</v>
+        <v>243</v>
       </c>
       <c r="I5" t="s">
-        <v>239</v>
+        <v>244</v>
       </c>
       <c r="J5" t="s">
-        <v>226</v>
+        <v>231</v>
       </c>
       <c r="K5" t="s">
-        <v>240</v>
+        <v>245</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>241</v>
+        <v>246</v>
       </c>
       <c r="B6" t="s">
-        <v>242</v>
+        <v>247</v>
       </c>
       <c r="C6" t="s">
         <v>22</v>
       </c>
       <c r="D6" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="E6" t="s">
         <v>14</v>
@@ -3010,30 +3025,30 @@
         <v>23</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>243</v>
+        <v>248</v>
       </c>
       <c r="I6" t="s">
-        <v>46</v>
+        <v>230</v>
       </c>
       <c r="J6" t="s">
-        <v>226</v>
+        <v>231</v>
       </c>
       <c r="K6" t="s">
-        <v>227</v>
+        <v>232</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>244</v>
+        <v>249</v>
       </c>
       <c r="B7" t="s">
-        <v>245</v>
+        <v>250</v>
       </c>
       <c r="C7" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="D7" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="E7" t="s">
         <v>28</v>
@@ -3045,30 +3060,30 @@
         <v>16</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>246</v>
+        <v>251</v>
       </c>
       <c r="I7" t="s">
-        <v>46</v>
+        <v>230</v>
       </c>
       <c r="J7" t="s">
-        <v>226</v>
+        <v>231</v>
       </c>
       <c r="K7" t="s">
-        <v>227</v>
+        <v>232</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>247</v>
+        <v>252</v>
       </c>
       <c r="B8" t="s">
-        <v>46</v>
+        <v>230</v>
       </c>
       <c r="C8" t="s">
         <v>12</v>
       </c>
       <c r="D8" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="E8" t="s">
         <v>14</v>
@@ -3080,16 +3095,16 @@
         <v>29</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="I8" t="s">
-        <v>46</v>
+        <v>230</v>
       </c>
       <c r="J8" t="s">
-        <v>226</v>
+        <v>231</v>
       </c>
       <c r="K8" t="s">
-        <v>227</v>
+        <v>232</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Swap round 2: Turbostart out (pre-Series A on re-check), BEENEXT in
- scripts/roundup-lookup.ts: a year of Inc42 + Entrackr weekly roundups
  (72 articles, Tavily only) -> 66 logistics rounds -> 2 B2B logistics
  software seed deals; 1 new (BEENEXT led CREST pre-seed).
- lib/rubric.ts: shared rubric for both discovery scripts.
- scripts/recheck-swapins.ts: Turbostart and Chiratae fail (pre-Series A);
  Picus/Wavemaker unverifiable (evidence blocks bots) -> kept.
- apply-swap: per-round plans and undo (CSV + DB), no git checkout.
- docs/swap-log.md round 2 section; export refreshed.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/vc-list-export.xlsx
+++ b/data/vc-list-export.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="598" uniqueCount="253">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="609" uniqueCount="258">
   <si>
     <t>Firm</t>
   </si>
@@ -317,6 +317,18 @@
     <t>https://www.araliventures.in</t>
   </si>
   <si>
+    <t>BEENEXT</t>
+  </si>
+  <si>
+    <t>Dirk Van Quaquebeke</t>
+  </si>
+  <si>
+    <t>Rubric swap-in round 2 (score 41.5): led pre-seed in CREST (Automated inventory planning software; 2026-06-20)</t>
+  </si>
+  <si>
+    <t>https://www.beenext.com</t>
+  </si>
+  <si>
     <t>Better Capital</t>
   </si>
   <si>
@@ -530,6 +542,195 @@
     <t>https://titancapital.vc</t>
   </si>
   <si>
+    <t>Wavemaker Partners</t>
+  </si>
+  <si>
+    <t>Paul Santos</t>
+  </si>
+  <si>
+    <t>Rubric swap-in (score 23.7): led pre-seed in Confluxe (Platform providing market entry strategy, digital commerce, merchandising, and supply chain operations; 2026-03-11)</t>
+  </si>
+  <si>
+    <t>https://wavemaker.vc</t>
+  </si>
+  <si>
+    <t>YourNest Venture Capital</t>
+  </si>
+  <si>
+    <t>Girish Shivani</t>
+  </si>
+  <si>
+    <t>Rubric swap-in (score 42.4): led seed in CargoFL (logistics technology platform to optimize freight and supply chain operations; 2026-06-24)</t>
+  </si>
+  <si>
+    <t>https://yournest.in</t>
+  </si>
+  <si>
+    <t>100X.VC</t>
+  </si>
+  <si>
+    <t>Sanjay Mehta</t>
+  </si>
+  <si>
+    <t>P3</t>
+  </si>
+  <si>
+    <t>Active India seed fund (iSAFE structure)</t>
+  </si>
+  <si>
+    <t>https://www.100x.vc</t>
+  </si>
+  <si>
+    <t>Ankur Capital</t>
+  </si>
+  <si>
+    <t>Krishnan Neelakantan</t>
+  </si>
+  <si>
+    <t>Agritech/agri-supply-chain focus - adjacent</t>
+  </si>
+  <si>
+    <t>https://www.ankurcapital.com</t>
+  </si>
+  <si>
+    <t>Antler India</t>
+  </si>
+  <si>
+    <t>Nitin Sharma</t>
+  </si>
+  <si>
+    <t>Day-zero/pre-seed platform</t>
+  </si>
+  <si>
+    <t>https://www.antler.co</t>
+  </si>
+  <si>
+    <t>Eclipse Ventures</t>
+  </si>
+  <si>
+    <t>Lior Susan</t>
+  </si>
+  <si>
+    <t>Listed for logistics but industrial/hardware-heavy - likely adjacent, not B2B software</t>
+  </si>
+  <si>
+    <t>https://eclipse.capital</t>
+  </si>
+  <si>
+    <t>LDV Capital</t>
+  </si>
+  <si>
+    <t>Evan Nisselson</t>
+  </si>
+  <si>
+    <t>Listed among early-stage logistics funds (deep-tech/visual tech skew)</t>
+  </si>
+  <si>
+    <t>https://www.ldv.co</t>
+  </si>
+  <si>
+    <t>Navigate Ventures</t>
+  </si>
+  <si>
+    <t>Ivan Nikkhoo</t>
+  </si>
+  <si>
+    <t>Appears in Signal NFX supply-chain seed list (LA region); confirm still active</t>
+  </si>
+  <si>
+    <t>https://www.navigatevc.com</t>
+  </si>
+  <si>
+    <t>pi Ventures</t>
+  </si>
+  <si>
+    <t>Shubham Sandeep</t>
+  </si>
+  <si>
+    <t>Deep-tech/AI focus - likely thematic (AI) rather than logistics</t>
+  </si>
+  <si>
+    <t>https://www.piventures.in</t>
+  </si>
+  <si>
+    <t>Prologis Ventures</t>
+  </si>
+  <si>
+    <t>William O'Donnell</t>
+  </si>
+  <si>
+    <t>Global</t>
+  </si>
+  <si>
+    <t>Corporate VC of a warehousing REIT; track for thematic signals</t>
+  </si>
+  <si>
+    <t>https://www.prologis.com</t>
+  </si>
+  <si>
+    <t>Speciale Invest</t>
+  </si>
+  <si>
+    <t>Vishesh Rajaram</t>
+  </si>
+  <si>
+    <t>Deep-tech/space/robotics focus; Rs 600Cr Fund III (Aug 2025) - mostly adjacent for B2B SaaS</t>
+  </si>
+  <si>
+    <t>https://www.specialeinvest.com</t>
+  </si>
+  <si>
+    <t>TMV</t>
+  </si>
+  <si>
+    <t>Marina Hadjipateras</t>
+  </si>
+  <si>
+    <t>Listed among early-stage logistics funds</t>
+  </si>
+  <si>
+    <t>https://www.tmv.vc</t>
+  </si>
+  <si>
+    <t>Archived reason</t>
+  </si>
+  <si>
+    <t>Enrission India Capital</t>
+  </si>
+  <si>
+    <t>YUSUKE KAKIMOTO</t>
+  </si>
+  <si>
+    <t>Led Hexalog $4M seed (logistics tech, Jan 2026) - verify B2B software fit</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>yes</t>
+  </si>
+  <si>
+    <t>no verified website</t>
+  </si>
+  <si>
+    <t>Stride Ventures</t>
+  </si>
+  <si>
+    <t>Apoorva Sharma</t>
+  </si>
+  <si>
+    <t>Series A+ only</t>
+  </si>
+  <si>
+    <t>Top Logistics SaaS investor by deal count per Tracxn (LoadShare, Ripplr, LetsTransport, Intangles) - likely venture debt, so confirm it does equity seed before prioritising</t>
+  </si>
+  <si>
+    <t>https://strideventures.global</t>
+  </si>
+  <si>
+    <t>venture debt</t>
+  </si>
+  <si>
     <t>Turbostart</t>
   </si>
   <si>
@@ -542,193 +743,7 @@
     <t>https://turbostart.co</t>
   </si>
   <si>
-    <t>Wavemaker Partners</t>
-  </si>
-  <si>
-    <t>Paul Santos</t>
-  </si>
-  <si>
-    <t>Rubric swap-in (score 23.7): led pre-seed in Confluxe (Platform providing market entry strategy, digital commerce, merchandising, and supply chain operations; 2026-03-11)</t>
-  </si>
-  <si>
-    <t>https://wavemaker.vc</t>
-  </si>
-  <si>
-    <t>YourNest Venture Capital</t>
-  </si>
-  <si>
-    <t>Girish Shivani</t>
-  </si>
-  <si>
-    <t>Rubric swap-in (score 42.4): led seed in CargoFL (logistics technology platform to optimize freight and supply chain operations; 2026-06-24)</t>
-  </si>
-  <si>
-    <t>https://yournest.in</t>
-  </si>
-  <si>
-    <t>100X.VC</t>
-  </si>
-  <si>
-    <t>Sanjay Mehta</t>
-  </si>
-  <si>
-    <t>P3</t>
-  </si>
-  <si>
-    <t>Active India seed fund (iSAFE structure)</t>
-  </si>
-  <si>
-    <t>https://www.100x.vc</t>
-  </si>
-  <si>
-    <t>Ankur Capital</t>
-  </si>
-  <si>
-    <t>Krishnan Neelakantan</t>
-  </si>
-  <si>
-    <t>Agritech/agri-supply-chain focus - adjacent</t>
-  </si>
-  <si>
-    <t>https://www.ankurcapital.com</t>
-  </si>
-  <si>
-    <t>Antler India</t>
-  </si>
-  <si>
-    <t>Nitin Sharma</t>
-  </si>
-  <si>
-    <t>Day-zero/pre-seed platform</t>
-  </si>
-  <si>
-    <t>https://www.antler.co</t>
-  </si>
-  <si>
-    <t>Eclipse Ventures</t>
-  </si>
-  <si>
-    <t>Lior Susan</t>
-  </si>
-  <si>
-    <t>Listed for logistics but industrial/hardware-heavy - likely adjacent, not B2B software</t>
-  </si>
-  <si>
-    <t>https://eclipse.capital</t>
-  </si>
-  <si>
-    <t>LDV Capital</t>
-  </si>
-  <si>
-    <t>Evan Nisselson</t>
-  </si>
-  <si>
-    <t>Listed among early-stage logistics funds (deep-tech/visual tech skew)</t>
-  </si>
-  <si>
-    <t>https://www.ldv.co</t>
-  </si>
-  <si>
-    <t>Navigate Ventures</t>
-  </si>
-  <si>
-    <t>Ivan Nikkhoo</t>
-  </si>
-  <si>
-    <t>Appears in Signal NFX supply-chain seed list (LA region); confirm still active</t>
-  </si>
-  <si>
-    <t>https://www.navigatevc.com</t>
-  </si>
-  <si>
-    <t>pi Ventures</t>
-  </si>
-  <si>
-    <t>Shubham Sandeep</t>
-  </si>
-  <si>
-    <t>Deep-tech/AI focus - likely thematic (AI) rather than logistics</t>
-  </si>
-  <si>
-    <t>https://www.piventures.in</t>
-  </si>
-  <si>
-    <t>Prologis Ventures</t>
-  </si>
-  <si>
-    <t>William O'Donnell</t>
-  </si>
-  <si>
-    <t>Global</t>
-  </si>
-  <si>
-    <t>Corporate VC of a warehousing REIT; track for thematic signals</t>
-  </si>
-  <si>
-    <t>https://www.prologis.com</t>
-  </si>
-  <si>
-    <t>Speciale Invest</t>
-  </si>
-  <si>
-    <t>Vishesh Rajaram</t>
-  </si>
-  <si>
-    <t>Deep-tech/space/robotics focus; Rs 600Cr Fund III (Aug 2025) - mostly adjacent for B2B SaaS</t>
-  </si>
-  <si>
-    <t>https://www.specialeinvest.com</t>
-  </si>
-  <si>
-    <t>TMV</t>
-  </si>
-  <si>
-    <t>Marina Hadjipateras</t>
-  </si>
-  <si>
-    <t>Listed among early-stage logistics funds</t>
-  </si>
-  <si>
-    <t>https://www.tmv.vc</t>
-  </si>
-  <si>
-    <t>Archived reason</t>
-  </si>
-  <si>
-    <t>Enrission India Capital</t>
-  </si>
-  <si>
-    <t>YUSUKE KAKIMOTO</t>
-  </si>
-  <si>
-    <t>Led Hexalog $4M seed (logistics tech, Jan 2026) - verify B2B software fit</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>yes</t>
-  </si>
-  <si>
-    <t>no verified website</t>
-  </si>
-  <si>
-    <t>Stride Ventures</t>
-  </si>
-  <si>
-    <t>Apoorva Sharma</t>
-  </si>
-  <si>
-    <t>Series A+ only</t>
-  </si>
-  <si>
-    <t>Top Logistics SaaS investor by deal count per Tracxn (LoadShare, Ripplr, LetsTransport, Intangles) - likely venture debt, so confirm it does equity seed before prioritising</t>
-  </si>
-  <si>
-    <t>https://strideventures.global</t>
-  </si>
-  <si>
-    <t>venture debt</t>
+    <t>round 2: failed re-check: round is "pre-Series A", not pre-seed/seed (evidence: https://entrepreneur.economictimes.indiatimes.com/amp/news/funding/lawyered-secures-25-million-pre-series-a-funding-to-revolutionize-legal-solutions-for-indias-mobility-sector/130410540)</t>
   </si>
   <si>
     <t>Venture Highway</t>
@@ -1831,7 +1846,7 @@
         <v>15</v>
       </c>
       <c r="G21" t="s">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="H21" s="1" t="s">
         <v>103</v>
@@ -1863,7 +1878,7 @@
         <v>15</v>
       </c>
       <c r="G22" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="H22" s="1" t="s">
         <v>107</v>
@@ -1883,13 +1898,13 @@
         <v>110</v>
       </c>
       <c r="C23" t="s">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="D23" t="s">
         <v>82</v>
       </c>
       <c r="E23" t="s">
-        <v>28</v>
+        <v>14</v>
       </c>
       <c r="F23" t="s">
         <v>15</v>
@@ -1915,7 +1930,7 @@
         <v>114</v>
       </c>
       <c r="C24" t="s">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="D24" t="s">
         <v>82</v>
@@ -1927,7 +1942,7 @@
         <v>15</v>
       </c>
       <c r="G24" t="s">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="H24" s="1" t="s">
         <v>115</v>
@@ -1979,13 +1994,13 @@
         <v>122</v>
       </c>
       <c r="C26" t="s">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="D26" t="s">
         <v>82</v>
       </c>
       <c r="E26" t="s">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="F26" t="s">
         <v>15</v>
@@ -2011,7 +2026,7 @@
         <v>126</v>
       </c>
       <c r="C27" t="s">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="D27" t="s">
         <v>82</v>
@@ -2049,7 +2064,7 @@
         <v>82</v>
       </c>
       <c r="E28" t="s">
-        <v>28</v>
+        <v>14</v>
       </c>
       <c r="F28" t="s">
         <v>15</v>
@@ -2081,7 +2096,7 @@
         <v>82</v>
       </c>
       <c r="E29" t="s">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="F29" t="s">
         <v>15</v>
@@ -2107,7 +2122,7 @@
         <v>138</v>
       </c>
       <c r="C30" t="s">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="D30" t="s">
         <v>82</v>
@@ -2116,10 +2131,10 @@
         <v>14</v>
       </c>
       <c r="F30" t="s">
-        <v>34</v>
+        <v>15</v>
       </c>
       <c r="G30" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="H30" s="1" t="s">
         <v>139</v>
@@ -2148,16 +2163,16 @@
         <v>14</v>
       </c>
       <c r="F31" t="s">
-        <v>15</v>
+        <v>34</v>
       </c>
       <c r="G31" t="s">
         <v>29</v>
       </c>
       <c r="H31" s="1" t="s">
-        <v>111</v>
+        <v>143</v>
       </c>
       <c r="I31" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="J31" t="s">
         <v>19</v>
@@ -2165,19 +2180,19 @@
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B32" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C32" t="s">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="D32" t="s">
         <v>82</v>
       </c>
       <c r="E32" t="s">
-        <v>28</v>
+        <v>14</v>
       </c>
       <c r="F32" t="s">
         <v>15</v>
@@ -2186,7 +2201,7 @@
         <v>29</v>
       </c>
       <c r="H32" s="1" t="s">
-        <v>146</v>
+        <v>115</v>
       </c>
       <c r="I32" t="s">
         <v>147</v>
@@ -2203,13 +2218,13 @@
         <v>149</v>
       </c>
       <c r="C33" t="s">
-        <v>150</v>
+        <v>22</v>
       </c>
       <c r="D33" t="s">
         <v>82</v>
       </c>
       <c r="E33" t="s">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="F33" t="s">
         <v>15</v>
@@ -2218,10 +2233,10 @@
         <v>29</v>
       </c>
       <c r="H33" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="I33" t="s">
         <v>151</v>
-      </c>
-      <c r="I33" t="s">
-        <v>152</v>
       </c>
       <c r="J33" t="s">
         <v>19</v>
@@ -2229,13 +2244,13 @@
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
+        <v>152</v>
+      </c>
+      <c r="B34" t="s">
         <v>153</v>
       </c>
-      <c r="B34" t="s">
+      <c r="C34" t="s">
         <v>154</v>
-      </c>
-      <c r="C34" t="s">
-        <v>22</v>
       </c>
       <c r="D34" t="s">
         <v>82</v>
@@ -2247,7 +2262,7 @@
         <v>15</v>
       </c>
       <c r="G34" t="s">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="H34" s="1" t="s">
         <v>155</v>
@@ -2267,19 +2282,19 @@
         <v>158</v>
       </c>
       <c r="C35" t="s">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="D35" t="s">
         <v>82</v>
       </c>
       <c r="E35" t="s">
-        <v>28</v>
+        <v>14</v>
       </c>
       <c r="F35" t="s">
         <v>15</v>
       </c>
       <c r="G35" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="H35" s="1" t="s">
         <v>159</v>
@@ -2314,10 +2329,10 @@
         <v>29</v>
       </c>
       <c r="H36" s="1" t="s">
-        <v>111</v>
+        <v>163</v>
       </c>
       <c r="I36" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="J36" t="s">
         <v>19</v>
@@ -2325,10 +2340,10 @@
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="B37" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="C37" t="s">
         <v>12</v>
@@ -2337,7 +2352,7 @@
         <v>82</v>
       </c>
       <c r="E37" t="s">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="F37" t="s">
         <v>15</v>
@@ -2346,7 +2361,7 @@
         <v>29</v>
       </c>
       <c r="H37" s="1" t="s">
-        <v>166</v>
+        <v>115</v>
       </c>
       <c r="I37" t="s">
         <v>167</v>
@@ -2363,7 +2378,7 @@
         <v>169</v>
       </c>
       <c r="C38" t="s">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="D38" t="s">
         <v>82</v>
@@ -2407,7 +2422,7 @@
         <v>15</v>
       </c>
       <c r="G39" t="s">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="H39" s="1" t="s">
         <v>174</v>
@@ -2812,7 +2827,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K8"/>
+  <dimension ref="A1:K9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -2937,7 +2952,7 @@
         <v>239</v>
       </c>
       <c r="B4" t="s">
-        <v>230</v>
+        <v>240</v>
       </c>
       <c r="C4" t="s">
         <v>22</v>
@@ -2952,54 +2967,54 @@
         <v>15</v>
       </c>
       <c r="G4" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="I4" t="s">
-        <v>230</v>
+        <v>242</v>
       </c>
       <c r="J4" t="s">
         <v>231</v>
       </c>
       <c r="K4" t="s">
-        <v>232</v>
+        <v>243</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="B5" t="s">
-        <v>242</v>
+        <v>230</v>
       </c>
       <c r="C5" t="s">
         <v>22</v>
       </c>
       <c r="D5" t="s">
-        <v>186</v>
+        <v>82</v>
       </c>
       <c r="E5" t="s">
         <v>14</v>
       </c>
       <c r="F5" t="s">
-        <v>235</v>
+        <v>15</v>
       </c>
       <c r="G5" t="s">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="I5" t="s">
-        <v>244</v>
+        <v>230</v>
       </c>
       <c r="J5" t="s">
         <v>231</v>
       </c>
       <c r="K5" t="s">
-        <v>245</v>
+        <v>232</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
@@ -3019,7 +3034,7 @@
         <v>14</v>
       </c>
       <c r="F6" t="s">
-        <v>15</v>
+        <v>235</v>
       </c>
       <c r="G6" t="s">
         <v>23</v>
@@ -3028,39 +3043,39 @@
         <v>248</v>
       </c>
       <c r="I6" t="s">
-        <v>230</v>
+        <v>249</v>
       </c>
       <c r="J6" t="s">
         <v>231</v>
       </c>
       <c r="K6" t="s">
-        <v>232</v>
+        <v>250</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="B7" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="C7" t="s">
-        <v>215</v>
+        <v>22</v>
       </c>
       <c r="D7" t="s">
         <v>186</v>
       </c>
       <c r="E7" t="s">
-        <v>28</v>
+        <v>14</v>
       </c>
       <c r="F7" t="s">
         <v>15</v>
       </c>
       <c r="G7" t="s">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="I7" t="s">
         <v>230</v>
@@ -3074,28 +3089,28 @@
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="B8" t="s">
-        <v>230</v>
+        <v>255</v>
       </c>
       <c r="C8" t="s">
-        <v>12</v>
+        <v>215</v>
       </c>
       <c r="D8" t="s">
         <v>186</v>
       </c>
       <c r="E8" t="s">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="F8" t="s">
-        <v>34</v>
+        <v>15</v>
       </c>
       <c r="G8" t="s">
-        <v>29</v>
+        <v>16</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>207</v>
+        <v>256</v>
       </c>
       <c r="I8" t="s">
         <v>230</v>
@@ -3104,6 +3119,41 @@
         <v>231</v>
       </c>
       <c r="K8" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>257</v>
+      </c>
+      <c r="B9" t="s">
+        <v>230</v>
+      </c>
+      <c r="C9" t="s">
+        <v>12</v>
+      </c>
+      <c r="D9" t="s">
+        <v>186</v>
+      </c>
+      <c r="E9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F9" t="s">
+        <v>34</v>
+      </c>
+      <c r="G9" t="s">
+        <v>29</v>
+      </c>
+      <c r="H9" s="1" t="s">
+        <v>207</v>
+      </c>
+      <c r="I9" t="s">
+        <v>230</v>
+      </c>
+      <c r="J9" t="s">
+        <v>231</v>
+      </c>
+      <c r="K9" t="s">
         <v>232</v>
       </c>
     </row>

</xml_diff>